<commit_message>
feat: implement full WSJF scoring pipeline with sample data
Adds working ingest/score/rank/export tools, scoring prompt, sample
backlog with 10 items, dotenv support, and CLAUDE.md agent guidelines.
Switches to Haiku model for cost efficiency.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/sample_backlog.xlsx
+++ b/examples/sample_backlog.xlsx
@@ -1,34 +1,282 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
+  <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peterwolyniec/Desktop/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E6D08FF-94DA-5840-AE48-CF9964BB0EAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Feature Backlog" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
+  <si>
+    <t>Feature ID</t>
+  </si>
+  <si>
+    <t>Feature Name</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Business Value</t>
+  </si>
+  <si>
+    <t>Time Criticality</t>
+  </si>
+  <si>
+    <t>Risk Reduction / Opportunity Enablement</t>
+  </si>
+  <si>
+    <t>Job Duration</t>
+  </si>
+  <si>
+    <t>F-001</t>
+  </si>
+  <si>
+    <t>Automated Data Quality Scoring</t>
+  </si>
+  <si>
+    <t>Automatically scores incoming datasets across 12 quality dimensions (completeness, accuracy, consistency, timeliness, etc.) using an ML classifier trained on 4M+ labeled records. Each dataset receives a 0–100 quality score with drill-down explanations. Scores are refreshed every 15 minutes and surfaced in the pipeline monitoring UI. Teams can set threshold-based alerts to block low-quality data from entering production. Integrated with dbt, Airbyte, and Fivetran connectors out of the box.</t>
+  </si>
+  <si>
+    <t>Eliminates approximately 18 person-hours per month spent on manual data profiling and validation checks by data engineers. Reduces data incident tickets by an estimated 35%, saving ~$12,000/year in incident response costs for a mid-size team. Improves analyst trust in data, increasing self-serve BI adoption by 20% based on pilot cohort data.</t>
+  </si>
+  <si>
+    <t>High — data quality issues compound quickly; a 15-minute detection window is critical to prevent bad data from propagating to 50+ downstream consumers. Delivery by Q2 is required to support a planned migration to a new data warehouse in Q3.</t>
+  </si>
+  <si>
+    <t>Risk Reduction — mitigates the risk of revenue-impacting decisions being made on corrupted or incomplete data. In one documented customer case, a data quality failure led to a $220,000 misbilling event. Automated scoring provides a systematic defense layer across all ingested datasets.</t>
+  </si>
+  <si>
+    <t>3 sprints (6 weeks) — includes ML model training pipeline, scoring API, UI integration, dbt/Airbyte/Fivetran connector builds, and alert configuration module. 1-week buffer allocated for QA and data validation with 3 design partner customers.</t>
+  </si>
+  <si>
+    <t>F-002</t>
+  </si>
+  <si>
+    <t>AI-Powered Anomaly Detection</t>
+  </si>
+  <si>
+    <t>Deploys an unsupervised ML model (Isolation Forest + LSTM hybrid) that continuously monitors 500+ metrics across data pipelines and warehouses to surface statistically significant anomalies in near real-time. The system baselines 90 days of historical patterns per metric and auto-tunes sensitivity. Detected anomalies are ranked by estimated business impact and routed to the relevant team via Slack, PagerDuty, or email. Average detection latency is under 3 minutes from event occurrence.</t>
+  </si>
+  <si>
+    <t>Reduces mean time to detect (MTTD) data incidents from an average of 4.2 hours to under 10 minutes, preventing an estimated 3–5 SLA breaches per month valued at $8,000–$25,000 each. Teams save approximately 22 person-hours per month previously spent on manual monitoring and on-call investigation.</t>
+  </si>
+  <si>
+    <t>Critical — every hour of delayed anomaly detection increases the blast radius of a data incident exponentially. Real-time monitoring is table-stakes for customers with sub-4-hour data SLAs. Required for enterprise tier launch in Q1.</t>
+  </si>
+  <si>
+    <t>Risk Reduction + Opportunity Enablement — reduces operational risk of undetected pipeline failures silently corrupting dashboards and ML feature stores. Also positions the platform as an enterprise-grade observability solution, unlocking the $500K+ ACV segment.</t>
+  </si>
+  <si>
+    <t>4 sprints (8 weeks) — model training and validation (2 weeks), real-time streaming integration (2 weeks), alert routing and notification framework (2 weeks), UI and explainability layer (2 weeks). Requires ML Eng, Data Eng, and Front-End resources in parallel.</t>
+  </si>
+  <si>
+    <t>F-003</t>
+  </si>
+  <si>
+    <t>Natural Language Query Interface</t>
+  </si>
+  <si>
+    <t>Enables business users to query any connected data warehouse using plain English sentences, which are translated to SQL via a fine-tuned code-generation LLM. The interface supports follow-up clarification prompts, auto-corrects ambiguous entity references, and logs all generated queries for auditability. Supports Snowflake, BigQuery, Redshift, and Databricks. A feedback loop allows data teams to rate query accuracy, continuously improving the model. No SQL knowledge required from end users.</t>
+  </si>
+  <si>
+    <t>Eliminates an estimated 30 ad-hoc data requests per analyst per month and frees up approximately 15 data engineer hours per month. Accelerates insight-to-decision cycles from 2–3 days to under 10 minutes for routine queries. Widens the addressable user base by ~10x per organization.</t>
+  </si>
+  <si>
+    <t>Medium — business stakeholders have been requesting self-serve query capabilities for 2+ quarters. Delay increases risk of teams building shadow analytics tools outside the platform.</t>
+  </si>
+  <si>
+    <t>Opportunity Enablement — dramatically widens the addressable user base beyond data professionals to include ~10x more business users per organization. Increases platform stickiness and drives seat expansion revenue. Positions product competitively against BI tools entering conversational analytics.</t>
+  </si>
+  <si>
+    <t>5 sprints (10 weeks) — LLM integration and prompt engineering (2 weeks), SQL generation accuracy benchmarking against 500-query test suite (2 weeks), warehouse connector development (3 weeks), feedback loop and UI (3 weeks). Accuracy target: &gt;90% on benchmark before GA.</t>
+  </si>
+  <si>
+    <t>F-004</t>
+  </si>
+  <si>
+    <t>Predictive Pipeline Failure Alerts</t>
+  </si>
+  <si>
+    <t>Uses time-series forecasting (Prophet + XGBoost ensemble) to predict pipeline failures up to 6 hours in advance with 87% precision. Monitors 30+ pipeline health signals including job duration variance, upstream data volume shifts, and API error rate trends. When a failure is predicted, the system auto-generates a root cause hypothesis and suggested remediation steps. Reduces mean time to resolution (MTTR) by surfacing issues before they cascade into downstream SLA breaches.</t>
+  </si>
+  <si>
+    <t>Prevents an estimated 4 pipeline failures per month from reaching production. Each failure averted saves an average of 6 hours of engineer remediation time and $5,000 in delayed business reporting costs. Reduces total on-call burden by approximately 25 hours per month across the data engineering team.</t>
+  </si>
+  <si>
+    <t>High — pipeline failures during month-end reporting periods carry disproportionate business impact. Predictive alerting must be in place before the fiscal Q3 close cycle to protect revenue-critical reporting workflows.</t>
+  </si>
+  <si>
+    <t>Risk Reduction — directly reduces the probability and impact of pipeline SLA breaches, which are the primary driver of customer churn in the data infrastructure category. Customers with critical financial or operational pipelines represent 70% of ARR.</t>
+  </si>
+  <si>
+    <t>3 sprints (6 weeks) — forecasting model development and backtesting (3 weeks), health signal ingestion pipeline (1 week), root cause hypothesis engine (1 week), notification and UI integration (1 week). Parallel with anomaly detection team to share signal infrastructure.</t>
+  </si>
+  <si>
+    <t>F-005</t>
+  </si>
+  <si>
+    <t>Auto-Schema Drift Detection</t>
+  </si>
+  <si>
+    <t>Continuously compares incoming data schemas against registered baselines and classifies drift events into breaking, non-breaking, and informational categories using a rules engine augmented by ML. Sends alerts within 90 seconds of a schema change being detected. Provides a visual diff view showing added, removed, and modified columns alongside impact analysis across 100+ downstream assets. Integrates directly into CI/CD pipelines to block deployments when breaking drift is identified.</t>
+  </si>
+  <si>
+    <t>Catches breaking schema changes before they propagate to downstream dashboards and models, preventing an estimated 8 downstream breakages per month — each averaging 3.5 hours to diagnose and fix. Total time savings of approximately 28 person-hours per month. Reduces data downtime visible to business stakeholders by an estimated 60%.</t>
+  </si>
+  <si>
+    <t>Critical — schema drift is the #1 root cause of data incidents reported by customers. Every week without this feature represents ongoing exposure to breaking changes that can silently corrupt BI dashboards.</t>
+  </si>
+  <si>
+    <t>Risk Reduction — schema drift is the leading cause of silent data failures, which are significantly more damaging than noisy failures because they go undetected. Also reduces dependency on tribal knowledge about upstream data contracts.</t>
+  </si>
+  <si>
+    <t>2 sprints (4 weeks) — schema registry integration (1 week), diff engine and classification rules (1 week), visual diff UI (1 week), CI/CD webhook integration (1 week). Relatively contained scope; accelerated timeline justified by high criticality.</t>
+  </si>
+  <si>
+    <t>F-006</t>
+  </si>
+  <si>
+    <t>LLM-Assisted Report Generation</t>
+  </si>
+  <si>
+    <t>Leverages a Claude-powered generation layer to automatically draft executive summaries, data narratives, and insight reports from structured query results. Users provide a natural language brief (e.g., 'summarize Q2 churn trends by region'), and the system retrieves relevant data, generates a 300–500 word narrative with embedded charts, and delivers it in PDF or Notion format. Drafts are produced in under 90 seconds. Supports custom brand tone guidelines via a style configuration file.</t>
+  </si>
+  <si>
+    <t>Reduces report production time from an average of 4 hours per report to under 10 minutes, saving approximately 20 person-hours per analyst per month across teams generating 5+ reports weekly. Estimated annual productivity value of $48,000 for a 5-person analytics team at a blended hourly rate of $80.</t>
+  </si>
+  <si>
+    <t>Medium — primarily an efficiency gain rather than a risk mitigation. However, the feature is referenced in 40% of active sales opportunities as a 'must-have' before signing.</t>
+  </si>
+  <si>
+    <t>Opportunity Enablement — unlocks a new use case category (automated narrative intelligence) that expands the platform's value proposition into executive reporting workflows. Creates a wedge into the office of the CFO and CMO, where the platform currently has low penetration.</t>
+  </si>
+  <si>
+    <t>3 sprints (6 weeks) — LLM generation layer and prompt templating (2 weeks), data retrieval and chart embedding pipeline (2 weeks), PDF/Notion export integration (1 week), brand style configuration (1 week). Leverages existing Claude API integration in platform.</t>
+  </si>
+  <si>
+    <t>F-007</t>
+  </si>
+  <si>
+    <t>Real-Time Cost Attribution Dashboard</t>
+  </si>
+  <si>
+    <t>Provides a live, drill-down dashboard that attributes cloud data infrastructure costs (compute, storage, egress) to individual teams, pipelines, users, and business domains with 95%+ tagging accuracy. Refreshes every 10 minutes using billing API integrations with AWS, GCP, and Azure. Surfaces cost anomalies, month-over-month trends, and projected spend forecasts with 30-day lookahead. Enables FinOps teams to set budget alerts and chargeback reports per department without manual spreadsheet work.</t>
+  </si>
+  <si>
+    <t>Enables an average 18% cloud cost reduction within 90 days through idle resource cleanup and query optimization. Eliminates approximately 12 person-hours per month of manual FinOps reporting. Organizations in the beta program recovered an average of $34,000 in the first quarter post-deployment.</t>
+  </si>
+  <si>
+    <t>High — cloud data cost overruns are a top-3 pain point for 65% of surveyed customers. FinOps initiatives at target enterprises are actively budgeting for Q2, making this the optimal window to capture the market need.</t>
+  </si>
+  <si>
+    <t>Opportunity Enablement + Risk Reduction — enables customers to justify and protect their data infrastructure budget by demonstrating ROI with precision. Opens door to FinOps-focused buyers as a new ICP segment.</t>
+  </si>
+  <si>
+    <t>4 sprints (8 weeks) — billing API integrations for AWS/GCP/Azure (3 weeks), tagging and attribution engine (2 weeks), dashboard UI and drill-down views (2 weeks), budget alert and chargeback report module (1 week).</t>
+  </si>
+  <si>
+    <t>F-008</t>
+  </si>
+  <si>
+    <t>Federated Query Optimizer</t>
+  </si>
+  <si>
+    <t>Optimizes federated queries spanning multiple data sources (e.g., Snowflake + PostgreSQL + S3) by intelligently rewriting execution plans to minimize data movement and compute cost. Uses a learned cost model trained on 10M+ historical query executions to select the optimal execution engine and pushdown strategy. Average query runtime reduction of 42% observed in beta testing across 50 enterprise customers. Fully transparent — users can inspect the rewrite logic via an explain plan UI.</t>
+  </si>
+  <si>
+    <t>Reduces average federated query execution time by 42%, cutting compute costs by an estimated 30% for high-volume workloads. For a company running 50,000 federated queries per month at $0.005/query average cost, this yields ~$750/month in direct savings. Data scientists reclaim approximately 10 hours per month previously lost waiting on slow cross-source queries.</t>
+  </si>
+  <si>
+    <t>Medium — two enterprise prospects have listed federated query performance as a blocker to upgrading from Standard to Enterprise tier, representing $180,000 ARR.</t>
+  </si>
+  <si>
+    <t>Opportunity Enablement — removes a key technical barrier to adopting multi-cloud and hybrid data architectures. Enables enterprises to consolidate query workloads onto the platform. Supports expansion into the $4.2B federated data management market.</t>
+  </si>
+  <si>
+    <t>5 sprints (10 weeks) — query plan analysis and rewrite engine (4 weeks), learned cost model training on historical query data (2 weeks), explain plan UI (2 weeks), performance benchmarking with enterprise beta customers (2 weeks). Highest technical complexity of the roadmap batch.</t>
+  </si>
+  <si>
+    <t>F-009</t>
+  </si>
+  <si>
+    <t>Intelligent Data Lineage Mapper</t>
+  </si>
+  <si>
+    <t>Automatically traces the full lineage of every data asset — from raw ingestion through transformations to BI dashboards — across 20+ supported connectors. Builds a graph of 10,000+ node relationships and makes it searchable via a visual explorer. Supports impact analysis ('what breaks if I change this table?') and root cause tracing ('why did this metric change?'). Lineage graphs are updated within 5 minutes of any pipeline execution and exportable as JSON or SVG.</t>
+  </si>
+  <si>
+    <t>Reduces impact analysis time ahead of schema or pipeline changes from an average of 3 hours to under 15 minutes, saving approximately 20 person-hours per month. Cuts mean time to root cause (MTTRC) for metric anomalies from 5.5 hours to 45 minutes. Reduces risk of undocumented data dependencies causing silent failures in production BI assets.</t>
+  </si>
+  <si>
+    <t>High — data governance and compliance requirements are accelerating, particularly in financial services and healthcare verticals. Automated lineage is a prerequisite for several active compliance audit cycles among top-10 accounts.</t>
+  </si>
+  <si>
+    <t>Risk Reduction + Compliance Enablement — directly addresses data governance requirements under GDPR, CCPA, and HIPAA by providing documented data provenance. Enables customers to pass data audits without manual documentation efforts.</t>
+  </si>
+  <si>
+    <t>4 sprints (8 weeks) — graph ingestion pipeline across 20 connectors (4 weeks), graph database setup and query layer (2 weeks), visual explorer UI (1 week), impact analysis and root cause modules (1 week). Connector work can be parallelized across 2 engineers.</t>
+  </si>
+  <si>
+    <t>F-010</t>
+  </si>
+  <si>
+    <t>AI Model Performance Monitor</t>
+  </si>
+  <si>
+    <t>Monitors deployed ML models across accuracy, drift, fairness, and data distribution metrics in real time. Calculates PSI (Population Stability Index) and SHAP-based feature importance shifts daily and raises alerts when model degradation is detected. Supports champion/challenger comparisons and auto-triggers retraining workflows when performance drops below configurable thresholds. Covers 15 model frameworks including scikit-learn, XGBoost, TensorFlow, and PyTorch. Provides a compliance-ready audit trail for all model versions.</t>
+  </si>
+  <si>
+    <t>Detects model degradation an average of 18 days earlier than manual review processes, preventing business costs of $15,000–$60,000 per incident from acting on stale predictions. Saves approximately 16 person-hours per month in manual monitoring tasks. Provides the audit trail required for AI governance compliance (EU AI Act, SR 11-7), avoiding potential regulatory risk.</t>
+  </si>
+  <si>
+    <t>Critical — EU AI Act enforcement begins August 2026, requiring documented model monitoring for high-risk AI systems. Customers in regulated industries face legal exposure without an automated monitoring and audit trail solution.</t>
+  </si>
+  <si>
+    <t>Risk Reduction + Regulatory Compliance — provides a documented, automated defense against model risk management failures. Also an Opportunity Enabler — the only platform in the mid-market segment offering built-in model governance at this price point.</t>
+  </si>
+  <si>
+    <t>3 sprints (6 weeks) — metric calculation engine (PSI, SHAP) for 15 frameworks (3 weeks), alert and retraining trigger system (1 week), champion/challenger comparison UI (1 week), audit trail and compliance export module (1 week).</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
       <color theme="1"/>
-      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -46,81 +294,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -199,6 +394,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -233,6 +429,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -267,20 +464,16 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -402,38 +595,317 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="30.83203125" customWidth="1"/>
+    <col min="3" max="7" width="40.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
+    <row r="1" spans="1:7" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="130" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="130" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="130" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="130" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="130" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="130" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="130" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="130" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="130" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="130" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>76</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:G11" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>